<commit_message>
Fix pricing false positives
</commit_message>
<xml_diff>
--- a/data/providers.xlsx
+++ b/data/providers.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>oes UX design consulting cost? Rates typically fall between $50 per hour and a multiple of that. Small projects; our and a multiple of that. Small projects can begin around $5,000 for project based pricing, while bigger</t>
+          <t>y fall between $50 per hour and a multip; n begin around $5,000 for project based</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Studies Coalition's SEO grew a niche jeweler's revenue from $160k/mo to $315k/mo in a year Coalition grew le; ition's SEO grew a niche jeweler's revenue from $160k/mo to $315k/mo in a year Coalition grew leads for Leas; adgen costs 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's se; 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's service Review; 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's service 4.8 GO</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
@@ -997,14 +997,10 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="AI3" s="2" t="inlineStr">
-        <is>
-          <t>https://coalitiontechnologies.com</t>
-        </is>
-      </c>
+      <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK3" s="2" t="inlineStr">
@@ -1014,12 +1010,12 @@
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>The agency cites over 800 client case studies, including growing a fashion ecommerce brand by $6M+ and increasing Lease Advisors' leads by 400%. Features verified portfolio case studies and publishes verified rates.</t>
+          <t>The agency cites over 800 client case studies, including growing a fashion ecommerce brand by $6M+ and increasing Lease Advisors' leads by 400%. Features verified portfolio case studies.</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>Direct contact email not displayed.</t>
+          <t>Pricing not publicly listed on the site. Direct contact email not displayed.</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1081,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>loring Continue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's yo; ng Continue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your r; tinue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in; What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in the c; your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in the company?</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1174,14 +1170,10 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="AI4" s="2" t="inlineStr">
-        <is>
-          <t>https://octet.design</t>
-        </is>
-      </c>
+      <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK4" s="2" t="inlineStr">
@@ -1191,12 +1183,12 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>The studio showcases a portfolio of 48 projects across sectors like SaaS, Enterprise, and FinTech, including specific work for clients like Trackier, Nirvana, and Survey2Connect. Features verified portfolio case studies and publishes verified rates.</t>
+          <t>The studio showcases a portfolio of 48 projects across sectors like SaaS, Enterprise, and FinTech, including specific work for clients like Trackier, Nirvana, and Survey2Connect. Features verified portfolio case studies.</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>Business location not confirmed in public structured data.</t>
+          <t>Pricing not publicly listed on the site. Business location not confirmed in public structured data.</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1419,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>inuous design QA. End to end From Design to Code Purchase | $79 AI MY Approach Work Process 01 Defining</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1516,14 +1508,10 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="AI6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.uxistudio.com</t>
-        </is>
-      </c>
+      <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK6" s="2" t="inlineStr">
@@ -1533,12 +1521,12 @@
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
-          <t>Ron Shenkar is a Senior Product Designer with 10 years of experience designing complex B2B platforms, specifically in cybersecurity and AI-enabled products. Features verified portfolio case studies and publishes verified rates.</t>
+          <t>Ron Shenkar is a Senior Product Designer with 10 years of experience designing complex B2B platforms, specifically in cybersecurity and AI-enabled products. Features verified portfolio case studies.</t>
         </is>
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>Noted concern: The 'Who We Are' section lists generic names like 'UX Ninja' and 'PR Goddess' which appear to be placeholder text or fictional personas.. Business location not confirmed in public structured data.</t>
+          <t>Pricing not publicly listed on the site. Noted concern: The 'Who We Are' section lists generic names like 'UX Ninja' and 'PR Goddess' which appear to be placeholder text or fictional personas.. Business location not confirmed in public structured data.</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1592,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>For smoother on-demand website maintenance needs. Starting $90/month Website Design Packages Get your busine; gn Packages Get your business up and running fast. Starting $990 eCommerce Website Design Packages Start; Packages Start selling online like big companies. Starting $1,200 Search Engine Optimization (SEO) Package; ackages Take your website higher in search engines Starting $350/month Managed Website Packages One package to; to design, develop, host &amp; maintain your website. Starting $99/month Top Factors That Affect Website Design</t>
+          <t>eeds. Starting $90/month Website Design; fast. Starting $990 eCommerce Website De; nies. Starting $1,200 Search Engine Opti</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -2984,7 +2972,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>live View Scope AI automation packages → Starting From USD $600 setup · $180/mo support Channels Web, Wh; ope AI automation packages → Starting From USD $600 setup · $180/mo support Channels Web, WhatsApp &amp; email; nger trust, and better lead conversion rates. Starting from INR 24,999 vs $8,000/mo developer save 97%+ View De; d better lead conversion rates. Starting from INR 24,999 vs $8,000/mo developer save 97%+ View Details SEO Se; under , Nouriva Wellness Verified Client ↑ CPL dropped from ₹4,200 → ₹2,050 "Cost per qualified lead halved</t>
+          <t>Starting From USD $300 / project Best F; rting From USD $300 / project Best For S; Starting From USD $600 [services] Digi</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -3161,7 +3149,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>to quality. Questions? Get in touch 40 hour plan per month $ 2600 /mo Perfect staff for your personality. Mee; omplimentary launch mtg. Get started 60 hour plan per month $ 3900 /mo Perfect staff for your personality. Mee; omplimentary launch mtg. Get started 80 hour plan per month $ 5200 /mo Perfect staff for your personality. Mee; mplimentary launch mtg. Get started 100 hour plan per month $ 6500 /mo Perfect staff for your personality. Mee; og writing, design and other specialist tasks are billed at $79/hr. Prices are based on monthly payment by</t>
+          <t>plan per month $ 2600 /mo Perfect staff; plan per month $ 3900 /mo Perfect staff; plan per month $ 5200 /mo Perfect staff</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
@@ -3507,7 +3495,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>e plan available with basic features. ☞ Paid plans start at $49/month , with additional features and customiz; satisfaction." - Daniel M . Pricing: ☞ Paid plans start at $49 to $99 per month . 8. Antavo - Customer; action." - Daniel M . Pricing: ☞ Paid plans start at $49 to $99 per month . 8. Antavo - Customer Loyalty Redefine</t>
+          <t>plans start at $49/month , with addition; plans start at $49 to $99 per month . 8.; tart at $49 to $99 per month . 8. Antavo</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -3688,7 +3676,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>ntrepreneur Small task work to keep on top of a few things. $599 / mo 12 Hours of Task Work Per Month 1 User; n Up Grow Project work that goes beyond inbox &amp; scheduling. $899 / mo 20 Hours of Task Work Per Month 2 Users; Small Business Operational help for everyday business tasks $1,199 / mo 30 Hours of Task Work Per Month 3 Users; n Up Team Plan Built to handle the most demanding workloads $1,699 / mo 45 Hours of Task Work Per Month 4 Users; ncluded Sign Up Outbound – 6 Hour Plan Small outbound tasks $599 / mo 6 Hours of Outbound Work Per Month Sign</t>
+          <t>a few things. $599 / mo 12 Hours of Tas; &amp; scheduling. $899 / mo 20 Hours of Tas; business tasks $1,199 / mo 30 Hours of T</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -4392,7 +4380,7 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>sults speak for themselves: Our clients have generated over £45 million in combined revenue in the last</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -4477,14 +4465,10 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="AI23" s="2" t="inlineStr">
-        <is>
-          <t>https://theaiautomationagency.ai</t>
-        </is>
-      </c>
+      <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK23" s="2" t="inlineStr">
@@ -4494,12 +4478,12 @@
       </c>
       <c r="AL23" s="2" t="inlineStr">
         <is>
-          <t>The agency claims their clients have generated over £45 million in combined revenue in the last two years through their implemented strategies. Publishes verified rates.</t>
+          <t>The agency claims their clients have generated over £45 million in combined revenue in the last two years through their implemented strategies.</t>
         </is>
       </c>
       <c r="AM23" s="2" t="inlineStr">
         <is>
-          <t>Noted concern: Vague 'money back guarantee' without defined terms. Business location not confirmed in public structured data.</t>
+          <t>Pricing not publicly listed on the site. Noted concern: Vague 'money back guarantee' without defined terms. Business location not confirmed in public structured data.</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4545,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>100% Client Satisfaction 24/7 Support Available Starting at ₹10,000 Mobile App Development We build native a; ifications &amp; Deep Linking Explore 46+ locations Starting at ₹6,000 Website Development We design and build; Coding for Technical SEO Explore 46+ locations Starting at ₹30,000 Software Development We build custom sof; p API &amp; SMS Notifications Explore 46+ locations Starting at ₹8,000 UI/UX Design Research-driven interface d; ems &amp; Component Libraries Explore 46+ locations Starting at ₹8,000 SEO Services Rank higher on Google and t</t>
+          <t>le Starting at ₹10,000 Mobile App Develo; ns Starting at ₹6,000 Website Developmen; ns Starting at ₹30,000 Software Developm</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -4907,7 +4891,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>s · Don't want to build it yourself? We'll set it up — from $199 → Your favorite agent. A whole new set o; 2 The new iPhone lineup All Pro Air 9:41 iPhone 17 Pro From $1,099 Shop now iPhone Air From $999 iPhone 17; Air 9:41 iPhone 17 Pro From $1,099 Shop now iPhone Air From $999 iPhone 17 From $799 One AI automation pl; ro From $1,099 Shop now iPhone Air From $999 iPhone 17 From $799 One AI automation platform. No trade-off; cross — or have our team rebuild and run them for you, from $199. Talk to us Scale without the bill shock</t>
+          <t>t it up — from $199 → Your favorite agen; for you, from $199. Talk to us Scale wi</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
@@ -5080,7 +5064,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>ing Packages for Mumbai Businesses Starter Small businesses ₹15,000 /mo ✓ SEO Optimization ✓ Social Media (2 pl</t>
+          <t>all businesses ₹15,000 /mo ✓ SEO Optimiz</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
@@ -5929,7 +5913,7 @@
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>00 contacts 500 contacts (6,000 emails) Cheapest Plan Price $25/month $29/month $9/month $13/month $15/month; s 500 contacts (6,000 emails) Cheapest Plan Price $25/month $29/month $9/month $13/month $15/month $9.99/mont; acts (6,000 emails) Cheapest Plan Price $25/month $29/month $9/month $13/month $15/month $9.99/month $15.58/; 00 emails) Cheapest Plan Price $25/month $29/month $9/month $13/month $15/month $9.99/month $15.58/month $9/m; Cheapest Plan Price $25/month $29/month $9/month $13/month $15/month $9.99/month $15.58/month $9/month $39/m</t>
+          <t>est Plan Price $25/month $29/month $9/mo; rice $25/month $29/month $9/month $13/mo; onth $29/month $9/month $13/month $15/mo</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr"/>
@@ -6782,7 +6766,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>them globally. $299 /month Global Payrol; urance agency. $2,349 /month Everything; rvice demands. $3,449 /month High-Volume</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr"/>
@@ -6859,10 +6843,14 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="AI37" s="2" t="inlineStr"/>
+      <c r="AI37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.agencyva.com</t>
+        </is>
+      </c>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="AK37" s="2" t="inlineStr">
@@ -6872,12 +6860,12 @@
       </c>
       <c r="AL37" s="2" t="inlineStr">
         <is>
-          <t>The provider claims to have placed thousands of virtual assistants and hundreds of licensed insurance professionals.</t>
+          <t>The provider claims to have placed thousands of virtual assistants and hundreds of licensed insurance professionals Publishes verified rates.</t>
         </is>
       </c>
       <c r="AM37" s="2" t="inlineStr">
         <is>
-          <t>Pricing not publicly listed on the site. Direct contact email not displayed.</t>
+          <t>Direct contact email not displayed.</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8114,7 @@
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>e and location. Generally, you should expect to pay between $30 and $100 an hour. Again, prices can be m; cation. Generally, you should expect to pay between $30 and $100 an hour. Again, prices can be more or le; fer an all-inclusive service package and may charge between $2,000 and $10,000+ to set up a fully functioni; inclusive service package and may charge between $2,000 and $10,000+ to set up a fully functioning Shopify; d complexity in the project. Freelancers may charge between $30 to $100 an hour. Agencies might charge b</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
@@ -8215,14 +8203,10 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="AI45" s="2" t="inlineStr">
-        <is>
-          <t>https://bloomagency.in</t>
-        </is>
-      </c>
+      <c r="AI45" s="2" t="inlineStr"/>
       <c r="AJ45" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK45" s="2" t="inlineStr">
@@ -8232,12 +8216,12 @@
       </c>
       <c r="AL45" s="2" t="inlineStr">
         <is>
-          <t>Established provider offering Search Engine Optimization, Pay Per Click, Social Media Marketing based in India. Publishes verified rates.</t>
+          <t>Established provider offering Search Engine Optimization, Pay Per Click, Social Media Marketing based in India.</t>
         </is>
       </c>
       <c r="AM45" s="2" t="inlineStr">
         <is>
-          <t>Noted concern: No concrete case studies or client names provided. Limited verified case studies or client references in public crawl.</t>
+          <t>Pricing not publicly listed on the site. Noted concern: No concrete case studies or client names provided. Limited verified case studies or client references in public crawl.</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9489,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>oes UX design consulting cost? Rates typically fall between $50 per hour and a multiple of that. Small projects; our and a multiple of that. Small projects can begin around $5,000 for project based pricing, while bigger</t>
+          <t>y fall between $50 per hour and a multip; n begin around $5,000 for project based</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -9682,7 +9666,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Studies Coalition's SEO grew a niche jeweler's revenue from $160k/mo to $315k/mo in a year Coalition grew le; ition's SEO grew a niche jeweler's revenue from $160k/mo to $315k/mo in a year Coalition grew leads for Leas; adgen costs 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's se; 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's service Review; 60% while increasing leads 400%+ 1ink grew from $525k/mo to $918k/mo in a year of Coalition's service 4.8 GO</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
@@ -9767,14 +9751,10 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="AI3" s="2" t="inlineStr">
-        <is>
-          <t>https://coalitiontechnologies.com</t>
-        </is>
-      </c>
+      <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK3" s="2" t="inlineStr">
@@ -9784,12 +9764,12 @@
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>The agency cites over 800 client case studies, including growing a fashion ecommerce brand by $6M+ and increasing Lease Advisors' leads by 400%. Features verified portfolio case studies and publishes verified rates.</t>
+          <t>The agency cites over 800 client case studies, including growing a fashion ecommerce brand by $6M+ and increasing Lease Advisors' leads by 400%. Features verified portfolio case studies.</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>Direct contact email not displayed.</t>
+          <t>Pricing not publicly listed on the site. Direct contact email not displayed.</t>
         </is>
       </c>
     </row>
@@ -9855,7 +9835,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>loring Continue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's yo; ng Continue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your r; tinue What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in; What's your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in the c; your budget range? * Select budget &lt; $5k $5k - $15k $15k - $50k $50k + What's your role in the company?</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -9944,14 +9924,10 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="AI4" s="2" t="inlineStr">
-        <is>
-          <t>https://octet.design</t>
-        </is>
-      </c>
+      <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="AK4" s="2" t="inlineStr">
@@ -9961,12 +9937,12 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>The studio showcases a portfolio of 48 projects across sectors like SaaS, Enterprise, and FinTech, including specific work for clients like Trackier, Nirvana, and Survey2Connect. Features verified portfolio case studies and publishes verified rates.</t>
+          <t>The studio showcases a portfolio of 48 projects across sectors like SaaS, Enterprise, and FinTech, including specific work for clients like Trackier, Nirvana, and Survey2Connect. Features verified portfolio case studies.</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>Business location not confirmed in public structured data.</t>
+          <t>Pricing not publicly listed on the site. Business location not confirmed in public structured data.</t>
         </is>
       </c>
     </row>
@@ -10197,7 +10173,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>For smoother on-demand website maintenance needs. Starting $90/month Website Design Packages Get your busine; gn Packages Get your business up and running fast. Starting $990 eCommerce Website Design Packages Start; Packages Start selling online like big companies. Starting $1,200 Search Engine Optimization (SEO) Package; ackages Take your website higher in search engines Starting $350/month Managed Website Packages One package to; to design, develop, host &amp; maintain your website. Starting $99/month Top Factors That Affect Website Design</t>
+          <t>eeds. Starting $90/month Website Design; fast. Starting $990 eCommerce Website De; nies. Starting $1,200 Search Engine Opti</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -11050,7 +11026,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>100% Client Satisfaction 24/7 Support Available Starting at ₹10,000 Mobile App Development We build native a; ifications &amp; Deep Linking Explore 46+ locations Starting at ₹6,000 Website Development We design and build; Coding for Technical SEO Explore 46+ locations Starting at ₹30,000 Software Development We build custom sof; p API &amp; SMS Notifications Explore 46+ locations Starting at ₹8,000 UI/UX Design Research-driven interface d; ems &amp; Component Libraries Explore 46+ locations Starting at ₹8,000 SEO Services Rank higher on Google and t</t>
+          <t>le Starting at ₹10,000 Mobile App Develo; ns Starting at ₹6,000 Website Developmen; ns Starting at ₹30,000 Software Developm</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">

</xml_diff>